<commit_message>
vault backup: 2026-06-02 14:43:17
</commit_message>
<xml_diff>
--- a/26年中集环科工作区/精益工作区/年度精益活动计划表.xlsx
+++ b/26年中集环科工作区/精益工作区/年度精益活动计划表.xlsx
@@ -548,7 +548,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>2026年精益活动日历（6月-12月）  |  编制：企管部 王瑞俊  |  更新：2026-05-27</t>
+          <t>2026年精益活动日历（6月-12月）  |  编制：企管部 王瑞俊  |  更新：2026-05-28</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>2026年精益改善课题清单  |  更新：2026-05-27</t>
+          <t>2026年精益改善课题清单  |  更新：2026-05-28</t>
         </is>
       </c>
     </row>
@@ -2933,7 +2933,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>2026年精益KPI追踪表  |  更新：2026-05-27</t>
+          <t>2026年精益KPI追踪表  |  更新：2026-05-28</t>
         </is>
       </c>
     </row>
@@ -3773,7 +3773,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>2026年精益改善责任矩阵（RACI）  |  更新：2026-05-27  |  R=执行负责人 A=批准/问责 C=需咨询/协作 I=需知会</t>
+          <t>2026年精益改善责任矩阵（RACI）  |  更新：2026-05-28  |  R=执行负责人 A=批准/问责 C=需咨询/协作 I=需知会</t>
         </is>
       </c>
     </row>

</xml_diff>